<commit_message>
Add purchase batch delete and refresh purchase order template
</commit_message>
<xml_diff>
--- a/backend/app/templates/purchase_order_template.xlsx
+++ b/backend/app/templates/purchase_order_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ddalg\OneDrive\문서\카카오톡 받은 파일\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/16b59dc5d76a24f7/Desktop/회사 문서/양식/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6684FD34-00F0-4482-B5D5-17E1DDC84D88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AC7FBFE-0DA2-4885-ACDD-B4722B342A2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="64380" yWindow="7710" windowWidth="19125" windowHeight="10110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="발주서" sheetId="1" r:id="rId1"/>
@@ -55,9 +55,6 @@
     <t>도금</t>
   </si>
   <si>
-    <t>비고</t>
-  </si>
-  <si>
     <t xml:space="preserve">※ 비고 : </t>
   </si>
   <si>
@@ -95,11 +92,15 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>발  주  일  :</t>
+    <t xml:space="preserve">발  주  일  : </t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>납  기  일  :</t>
+    <t xml:space="preserve">납  기  일  : </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>발주처</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -266,12 +267,6 @@
   </cellStyleXfs>
   <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -333,12 +328,20 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="177" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -374,7 +377,7 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -384,7 +387,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="10"/>
-        <color rgb="FF333333"/>
+        <color rgb="FF222222"/>
         <name val="맑은 고딕"/>
         <family val="3"/>
         <charset val="129"/>
@@ -396,7 +399,7 @@
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -552,7 +555,85 @@
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF222222"/>
+        <name val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF222222"/>
+        <name val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF222222"/>
+        <name val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -582,7 +663,7 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
+        <b/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -592,7 +673,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="10"/>
-        <color rgb="FF222222"/>
+        <color rgb="FF333333"/>
         <name val="맑은 고딕"/>
         <family val="3"/>
         <charset val="129"/>
@@ -604,85 +685,7 @@
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF222222"/>
-        <name val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF222222"/>
-        <name val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF222222"/>
-        <name val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border>
@@ -762,13 +765,13 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>5</xdr:col>
-          <xdr:colOff>238125</xdr:colOff>
+          <xdr:colOff>247650</xdr:colOff>
           <xdr:row>0</xdr:row>
           <xdr:rowOff>219075</xdr:rowOff>
         </xdr:from>
         <xdr:to>
-          <xdr:col>11</xdr:col>
-          <xdr:colOff>9525</xdr:colOff>
+          <xdr:col>10</xdr:col>
+          <xdr:colOff>923925</xdr:colOff>
           <xdr:row>3</xdr:row>
           <xdr:rowOff>9525</xdr:rowOff>
         </xdr:to>
@@ -785,7 +788,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Sheet1!$B$2:$E$3" spid="_x0000_s1050"/>
+                  <a14:cameraTool cellRange="Sheet1!$B$2:$E$3" spid="_x0000_s1057"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -799,7 +802,7 @@
           </xdr:blipFill>
           <xdr:spPr bwMode="auto">
             <a:xfrm>
-              <a:off x="6638925" y="219075"/>
+              <a:off x="7248525" y="219075"/>
               <a:ext cx="2828925" cy="1009650"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -825,20 +828,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{12F0DFEC-E47A-4EA6-9494-1EC95216F28E}" name="표2" displayName="표2" ref="A5:K24" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
-  <autoFilter ref="A5:K24" xr:uid="{12F0DFEC-E47A-4EA6-9494-1EC95216F28E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{12F0DFEC-E47A-4EA6-9494-1EC95216F28E}" name="표2" displayName="표2" ref="A5:K23" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+  <autoFilter ref="A5:K23" xr:uid="{12F0DFEC-E47A-4EA6-9494-1EC95216F28E}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{DC64E7DD-D3AB-4C07-ADEE-71E86EAA1C3F}" name="품번" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{A2C399A9-D31D-4AFF-854A-6413F3A3C05C}" name="도번" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{F6C7AE50-A4AD-4109-9263-3CE98D0242BA}" name="품명" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{8647DA7E-7855-489B-8115-9564EC878706}" name="규격" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{45A2C5AD-5050-43A6-9063-35A4B3CD6956}" name="재질" dataDxfId="8"/>
-    <tableColumn id="12" xr3:uid="{4AE5F785-9888-4E51-B807-9561FB8D28C8}" name="완제품수량" dataDxfId="7" dataCellStyle="쉼표 [0]"/>
-    <tableColumn id="6" xr3:uid="{C206259F-BEB6-488C-B902-EF7877315B40}" name="단품_x000a_수량" dataDxfId="6" dataCellStyle="쉼표 [0]"/>
-    <tableColumn id="8" xr3:uid="{D99D1077-B437-46A3-9B22-0968F5AFA527}" name="열처리" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{16179CF6-C8BA-4BE2-BF6D-58316A045B8D}" name="용접" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{A7B32D29-392D-4669-8684-6675AAC7D2C3}" name="도금" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{71EA206A-302D-4413-BD38-B71BC09AD4C1}" name="비고" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{DC64E7DD-D3AB-4C07-ADEE-71E86EAA1C3F}" name="품번" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{A2C399A9-D31D-4AFF-854A-6413F3A3C05C}" name="도번" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{F6C7AE50-A4AD-4109-9263-3CE98D0242BA}" name="품명" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{8647DA7E-7855-489B-8115-9564EC878706}" name="규격" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{45A2C5AD-5050-43A6-9063-35A4B3CD6956}" name="재질" dataDxfId="6"/>
+    <tableColumn id="12" xr3:uid="{4AE5F785-9888-4E51-B807-9561FB8D28C8}" name="완제품수량" dataDxfId="5" dataCellStyle="쉼표 [0]"/>
+    <tableColumn id="6" xr3:uid="{C206259F-BEB6-488C-B902-EF7877315B40}" name="단품_x000a_수량" dataDxfId="4" dataCellStyle="쉼표 [0]"/>
+    <tableColumn id="8" xr3:uid="{D99D1077-B437-46A3-9B22-0968F5AFA527}" name="열처리" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{16179CF6-C8BA-4BE2-BF6D-58316A045B8D}" name="용접" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{A7B32D29-392D-4669-8684-6675AAC7D2C3}" name="도금" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{71EA206A-302D-4413-BD38-B71BC09AD4C1}" name="발주처" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="표 스타일 1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1129,345 +1132,333 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K24"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="19.5" customHeight="1" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K23"/>
+  <sheetFormatPr defaultColWidth="11.58203125" defaultRowHeight="19.5" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="2" width="11.875" style="4" customWidth="1"/>
-    <col min="3" max="3" width="23.625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="26.625" style="4" customWidth="1"/>
-    <col min="5" max="5" width="10" style="4" customWidth="1"/>
-    <col min="6" max="7" width="6.5" style="4" customWidth="1"/>
-    <col min="8" max="10" width="4.875" style="4" customWidth="1"/>
-    <col min="11" max="11" width="12.5" style="4" customWidth="1"/>
-    <col min="12" max="16384" width="11.625" style="4"/>
+    <col min="1" max="2" width="13.33203125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="25.5" style="2" customWidth="1"/>
+    <col min="4" max="4" width="29.58203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="10" style="2" customWidth="1"/>
+    <col min="6" max="7" width="6.5" style="2" customWidth="1"/>
+    <col min="8" max="8" width="5.5" style="2" customWidth="1"/>
+    <col min="9" max="10" width="4.83203125" style="2" customWidth="1"/>
+    <col min="11" max="11" width="12.5" style="2" customWidth="1"/>
+    <col min="12" max="16384" width="11.58203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="5"/>
-      <c r="D1" s="6" t="s">
+    <row r="1" spans="1:11" ht="36.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C1" s="3"/>
+      <c r="D1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I1" s="5"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+    </row>
+    <row r="2" spans="1:11" ht="36.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="D2" s="3"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+    </row>
+    <row r="3" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A3" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="I1" s="7"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-    </row>
-    <row r="2" spans="1:11" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D2" s="5"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="10"/>
-      <c r="K2" s="10"/>
-    </row>
-    <row r="3" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="24" t="s">
+      <c r="B3" s="22"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+    </row>
+    <row r="4" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="25"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-    </row>
-    <row r="4" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="26" t="s">
+      <c r="B4" s="22"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="12"/>
+    </row>
+    <row r="5" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A5" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I5" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="J5" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="K5" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="25"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="12"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="14"/>
-    </row>
-    <row r="5" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="E5" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="F5" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="G5" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="H5" s="17" t="s">
-        <v>4</v>
-      </c>
-      <c r="I5" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="J5" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="K5" s="15" t="s">
+    </row>
+    <row r="6" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="16"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="19"/>
+      <c r="J6" s="19"/>
+      <c r="K6" s="19"/>
+    </row>
+    <row r="7" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="16"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="19"/>
+    </row>
+    <row r="8" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A8" s="16"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
+      <c r="K8" s="19"/>
+    </row>
+    <row r="9" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A9" s="16"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19"/>
+    </row>
+    <row r="10" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A10" s="16"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="19"/>
+      <c r="J10" s="19"/>
+      <c r="K10" s="19"/>
+    </row>
+    <row r="11" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A11" s="16"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="19"/>
+      <c r="J11" s="19"/>
+      <c r="K11" s="19"/>
+    </row>
+    <row r="12" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A12" s="16"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="19"/>
+      <c r="I12" s="19"/>
+      <c r="J12" s="19"/>
+      <c r="K12" s="19"/>
+    </row>
+    <row r="13" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A13" s="16"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="19"/>
+      <c r="J13" s="19"/>
+      <c r="K13" s="19"/>
+    </row>
+    <row r="14" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A14" s="16"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="18"/>
+      <c r="H14" s="19"/>
+      <c r="I14" s="19"/>
+      <c r="J14" s="19"/>
+      <c r="K14" s="19"/>
+    </row>
+    <row r="15" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="16"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="19"/>
+      <c r="I15" s="19"/>
+      <c r="J15" s="19"/>
+      <c r="K15" s="19"/>
+    </row>
+    <row r="16" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A16" s="16"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="19"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
+    </row>
+    <row r="17" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="16"/>
+      <c r="B17" s="16"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="19"/>
+      <c r="I17" s="19"/>
+      <c r="J17" s="19"/>
+      <c r="K17" s="19"/>
+    </row>
+    <row r="18" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A18" s="16"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="19"/>
+      <c r="I18" s="19"/>
+      <c r="J18" s="19"/>
+      <c r="K18" s="19"/>
+    </row>
+    <row r="19" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A19" s="16"/>
+      <c r="B19" s="16"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="18"/>
+      <c r="H19" s="19"/>
+      <c r="I19" s="19"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="19"/>
+    </row>
+    <row r="20" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A20" s="16"/>
+      <c r="B20" s="16"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="19"/>
+      <c r="J20" s="19"/>
+      <c r="K20" s="19"/>
+    </row>
+    <row r="21" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A21" s="20"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="18"/>
+      <c r="G21" s="18"/>
+      <c r="H21" s="19"/>
+      <c r="I21" s="19"/>
+      <c r="J21" s="19"/>
+      <c r="K21" s="19"/>
+    </row>
+    <row r="22" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A22" s="20"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="18"/>
+      <c r="G22" s="18"/>
+      <c r="H22" s="19"/>
+      <c r="I22" s="19"/>
+      <c r="J22" s="19"/>
+      <c r="K22" s="19"/>
+    </row>
+    <row r="23" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A23" s="21" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="18"/>
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="21"/>
-      <c r="I6" s="21"/>
-      <c r="J6" s="21"/>
-      <c r="K6" s="21"/>
-    </row>
-    <row r="7" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="18"/>
-      <c r="B7" s="18"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="20"/>
-      <c r="H7" s="21"/>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
-      <c r="K7" s="21"/>
-    </row>
-    <row r="8" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="18"/>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="19"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="21"/>
-      <c r="I8" s="21"/>
-      <c r="J8" s="21"/>
-      <c r="K8" s="21"/>
-    </row>
-    <row r="9" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="18"/>
-      <c r="B9" s="18"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="21"/>
-      <c r="I9" s="21"/>
-      <c r="J9" s="21"/>
-      <c r="K9" s="21"/>
-    </row>
-    <row r="10" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="18"/>
-      <c r="B10" s="18"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="21"/>
-      <c r="I10" s="21"/>
-      <c r="J10" s="21"/>
-      <c r="K10" s="21"/>
-    </row>
-    <row r="11" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="18"/>
-      <c r="B11" s="18"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="21"/>
-      <c r="I11" s="21"/>
-      <c r="J11" s="21"/>
-      <c r="K11" s="21"/>
-    </row>
-    <row r="12" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="18"/>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="21"/>
-      <c r="I12" s="21"/>
-      <c r="J12" s="21"/>
-      <c r="K12" s="21"/>
-    </row>
-    <row r="13" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="18"/>
-      <c r="B13" s="18"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="21"/>
-      <c r="I13" s="21"/>
-      <c r="J13" s="21"/>
-      <c r="K13" s="21"/>
-    </row>
-    <row r="14" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="18"/>
-      <c r="B14" s="18"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="21"/>
-      <c r="I14" s="21"/>
-      <c r="J14" s="21"/>
-      <c r="K14" s="21"/>
-    </row>
-    <row r="15" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="18"/>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="21"/>
-      <c r="I15" s="21"/>
-      <c r="J15" s="21"/>
-      <c r="K15" s="21"/>
-    </row>
-    <row r="16" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="18"/>
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="21"/>
-      <c r="I16" s="21"/>
-      <c r="J16" s="21"/>
-      <c r="K16" s="21"/>
-    </row>
-    <row r="17" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="18"/>
-      <c r="B17" s="18"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="20"/>
-      <c r="H17" s="21"/>
-      <c r="I17" s="21"/>
-      <c r="J17" s="21"/>
-      <c r="K17" s="21"/>
-    </row>
-    <row r="18" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="18"/>
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="20"/>
-      <c r="H18" s="21"/>
-      <c r="I18" s="21"/>
-      <c r="J18" s="21"/>
-      <c r="K18" s="21"/>
-    </row>
-    <row r="19" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="18"/>
-      <c r="B19" s="18"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="21"/>
-      <c r="I19" s="21"/>
-      <c r="J19" s="21"/>
-      <c r="K19" s="21"/>
-    </row>
-    <row r="20" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="18"/>
-      <c r="B20" s="18"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="21"/>
-      <c r="I20" s="21"/>
-      <c r="J20" s="21"/>
-      <c r="K20" s="21"/>
-    </row>
-    <row r="21" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="18"/>
-      <c r="B21" s="18"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="20"/>
-      <c r="H21" s="21"/>
-      <c r="I21" s="21"/>
-      <c r="J21" s="21"/>
-      <c r="K21" s="21"/>
-    </row>
-    <row r="22" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="22"/>
-      <c r="B22" s="22"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="21"/>
-      <c r="F22" s="20"/>
-      <c r="G22" s="20"/>
-      <c r="H22" s="21"/>
-      <c r="I22" s="21"/>
-      <c r="J22" s="21"/>
-      <c r="K22" s="21"/>
-    </row>
-    <row r="23" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="22"/>
-      <c r="B23" s="22"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="21"/>
-      <c r="F23" s="20"/>
-      <c r="G23" s="20"/>
-      <c r="H23" s="21"/>
-      <c r="I23" s="21"/>
-      <c r="J23" s="21"/>
-      <c r="K23" s="21"/>
-    </row>
-    <row r="24" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="23" t="s">
-        <v>8</v>
-      </c>
-      <c r="B24" s="22"/>
-      <c r="C24" s="22"/>
-      <c r="D24" s="22"/>
-      <c r="E24" s="21"/>
-      <c r="F24" s="20"/>
-      <c r="G24" s="20"/>
-      <c r="H24" s="21"/>
-      <c r="I24" s="21"/>
-      <c r="J24" s="21"/>
-      <c r="K24" s="21"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="18"/>
+      <c r="G23" s="18"/>
+      <c r="H23" s="19"/>
+      <c r="I23" s="19"/>
+      <c r="J23" s="19"/>
+      <c r="K23" s="19"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.39370078740157483" bottom="0.78740157480314965" header="0.19685039370078741" footer="0.19685039370078741"/>
-  <pageSetup orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;G</oddFooter>
   </headerFooter>
@@ -1483,32 +1474,32 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F5BE80B-CF81-49E9-8E91-D91E022A6081}">
   <dimension ref="B1:E3"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="4.75" customWidth="1"/>
     <col min="3" max="5" width="10.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:5" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="2" t="s">
+    <row r="1" spans="2:5" ht="17.5" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="2" spans="2:5" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B2" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="2:5" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="3"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
+    </row>
+    <row r="3" spans="2:5" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B3" s="26"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1516,5 +1507,6 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Rename supplier to purchase company and simplify purchase batch UI
</commit_message>
<xml_diff>
--- a/backend/app/templates/purchase_order_template.xlsx
+++ b/backend/app/templates/purchase_order_template.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/16b59dc5d76a24f7/Desktop/회사 문서/양식/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AC7FBFE-0DA2-4885-ACDD-B4722B342A2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{2AC7FBFE-0DA2-4885-ACDD-B4722B342A2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2749398-88DE-4CEB-8EB4-91DBA058A033}"/>
   <bookViews>
-    <workbookView xWindow="64380" yWindow="7710" windowWidth="19125" windowHeight="10110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="4515" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="발주서" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>도번</t>
   </si>
@@ -71,23 +70,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>담당</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>검토</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>대표</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>결
-재</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>발  주  서</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -113,7 +95,7 @@
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="177" formatCode="yyyy\.mm\.dd"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -133,21 +115,6 @@
       <color theme="1"/>
       <name val="맑은 고딕"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="맑은 고딕"/>
-      <family val="3"/>
-      <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -235,7 +202,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -243,21 +210,6 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </left>
-      <right style="medium">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </right>
-      <top style="medium">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </top>
-      <bottom style="medium">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -265,83 +217,74 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="177" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -788,7 +731,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Sheet1!$B$2:$E$3" spid="_x0000_s1057"/>
+                  <a14:cameraTool cellRange="#REF!" spid="_x0000_s1059"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1135,324 +1078,324 @@
   <dimension ref="A1:K23"/>
   <sheetFormatPr defaultColWidth="11.58203125" defaultRowHeight="19.5" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="2" width="13.33203125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="25.5" style="2" customWidth="1"/>
-    <col min="4" max="4" width="29.58203125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="10" style="2" customWidth="1"/>
-    <col min="6" max="7" width="6.5" style="2" customWidth="1"/>
-    <col min="8" max="8" width="5.5" style="2" customWidth="1"/>
-    <col min="9" max="10" width="4.83203125" style="2" customWidth="1"/>
-    <col min="11" max="11" width="12.5" style="2" customWidth="1"/>
-    <col min="12" max="16384" width="11.58203125" style="2"/>
+    <col min="1" max="2" width="13.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="25.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="29.58203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="10" style="1" customWidth="1"/>
+    <col min="6" max="7" width="6.5" style="1" customWidth="1"/>
+    <col min="8" max="8" width="5.5" style="1" customWidth="1"/>
+    <col min="9" max="10" width="4.83203125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="11.58203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="36.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C1" s="3"/>
-      <c r="D1" s="4" t="s">
-        <v>15</v>
+      <c r="C1" s="2"/>
+      <c r="D1" s="3" t="s">
+        <v>11</v>
       </c>
-      <c r="I1" s="5"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
     </row>
     <row r="2" spans="1:11" ht="36.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D2" s="3"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
+      <c r="D2" s="2"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
     </row>
     <row r="3" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="23" t="s">
-        <v>16</v>
+      <c r="A3" s="22" t="s">
+        <v>12</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
+      <c r="B3" s="21"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
     </row>
     <row r="4" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="24" t="s">
-        <v>17</v>
+      <c r="A4" s="23" t="s">
+        <v>13</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="12"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="11"/>
     </row>
     <row r="5" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="14" t="s">
+      <c r="G5" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="15" t="s">
+      <c r="H5" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="I5" s="13" t="s">
+      <c r="I5" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="13" t="s">
+      <c r="J5" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="K5" s="13" t="s">
-        <v>18</v>
+      <c r="K5" s="12" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="16"/>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
+      <c r="A6" s="15"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
     </row>
     <row r="7" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="16"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="19"/>
+      <c r="A7" s="15"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="18"/>
     </row>
     <row r="8" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="16"/>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="19"/>
-      <c r="I8" s="19"/>
-      <c r="J8" s="19"/>
-      <c r="K8" s="19"/>
+      <c r="A8" s="15"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="18"/>
     </row>
     <row r="9" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="16"/>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="19"/>
-      <c r="I9" s="19"/>
-      <c r="J9" s="19"/>
-      <c r="K9" s="19"/>
+      <c r="A9" s="15"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="18"/>
+      <c r="J9" s="18"/>
+      <c r="K9" s="18"/>
     </row>
     <row r="10" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="16"/>
-      <c r="B10" s="16"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="19"/>
-      <c r="I10" s="19"/>
-      <c r="J10" s="19"/>
-      <c r="K10" s="19"/>
+      <c r="A10" s="15"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="18"/>
+      <c r="J10" s="18"/>
+      <c r="K10" s="18"/>
     </row>
     <row r="11" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="16"/>
-      <c r="B11" s="16"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="19"/>
-      <c r="I11" s="19"/>
-      <c r="J11" s="19"/>
-      <c r="K11" s="19"/>
+      <c r="A11" s="15"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="18"/>
+      <c r="J11" s="18"/>
+      <c r="K11" s="18"/>
     </row>
     <row r="12" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="16"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="19"/>
-      <c r="I12" s="19"/>
-      <c r="J12" s="19"/>
-      <c r="K12" s="19"/>
+      <c r="A12" s="15"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
+      <c r="J12" s="18"/>
+      <c r="K12" s="18"/>
     </row>
     <row r="13" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="16"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="19"/>
-      <c r="I13" s="19"/>
-      <c r="J13" s="19"/>
-      <c r="K13" s="19"/>
+      <c r="A13" s="15"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="18"/>
+      <c r="J13" s="18"/>
+      <c r="K13" s="18"/>
     </row>
     <row r="14" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="16"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="19"/>
-      <c r="I14" s="19"/>
-      <c r="J14" s="19"/>
-      <c r="K14" s="19"/>
+      <c r="A14" s="15"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="18"/>
+      <c r="J14" s="18"/>
+      <c r="K14" s="18"/>
     </row>
     <row r="15" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="16"/>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="18"/>
-      <c r="H15" s="19"/>
-      <c r="I15" s="19"/>
-      <c r="J15" s="19"/>
-      <c r="K15" s="19"/>
+      <c r="A15" s="15"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="18"/>
+      <c r="I15" s="18"/>
+      <c r="J15" s="18"/>
+      <c r="K15" s="18"/>
     </row>
     <row r="16" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="16"/>
-      <c r="B16" s="16"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="19"/>
-      <c r="J16" s="19"/>
-      <c r="K16" s="19"/>
+      <c r="A16" s="15"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="18"/>
+      <c r="I16" s="18"/>
+      <c r="J16" s="18"/>
+      <c r="K16" s="18"/>
     </row>
     <row r="17" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="16"/>
-      <c r="B17" s="16"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19"/>
-      <c r="J17" s="19"/>
-      <c r="K17" s="19"/>
+      <c r="A17" s="15"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="18"/>
+      <c r="J17" s="18"/>
+      <c r="K17" s="18"/>
     </row>
     <row r="18" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="16"/>
-      <c r="B18" s="16"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
-      <c r="J18" s="19"/>
-      <c r="K18" s="19"/>
+      <c r="A18" s="15"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="18"/>
+      <c r="J18" s="18"/>
+      <c r="K18" s="18"/>
     </row>
     <row r="19" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="16"/>
-      <c r="B19" s="16"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="19"/>
-      <c r="I19" s="19"/>
-      <c r="J19" s="19"/>
-      <c r="K19" s="19"/>
+      <c r="A19" s="15"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="18"/>
+      <c r="I19" s="18"/>
+      <c r="J19" s="18"/>
+      <c r="K19" s="18"/>
     </row>
     <row r="20" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="16"/>
-      <c r="B20" s="16"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="19"/>
-      <c r="J20" s="19"/>
-      <c r="K20" s="19"/>
+      <c r="A20" s="15"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="18"/>
+      <c r="J20" s="18"/>
+      <c r="K20" s="18"/>
     </row>
     <row r="21" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="20"/>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="18"/>
-      <c r="G21" s="18"/>
-      <c r="H21" s="19"/>
-      <c r="I21" s="19"/>
-      <c r="J21" s="19"/>
-      <c r="K21" s="19"/>
+      <c r="A21" s="19"/>
+      <c r="B21" s="19"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="18"/>
+      <c r="I21" s="18"/>
+      <c r="J21" s="18"/>
+      <c r="K21" s="18"/>
     </row>
     <row r="22" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="20"/>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="20"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="19"/>
-      <c r="I22" s="19"/>
-      <c r="J22" s="19"/>
-      <c r="K22" s="19"/>
+      <c r="A22" s="19"/>
+      <c r="B22" s="19"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="18"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="18"/>
+      <c r="I22" s="18"/>
+      <c r="J22" s="18"/>
+      <c r="K22" s="18"/>
     </row>
     <row r="23" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A23" s="21" t="s">
+      <c r="A23" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="19"/>
-      <c r="I23" s="19"/>
-      <c r="J23" s="19"/>
-      <c r="K23" s="19"/>
+      <c r="B23" s="19"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="18"/>
+      <c r="J23" s="18"/>
+      <c r="K23" s="18"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -1469,44 +1412,4 @@
     <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F5BE80B-CF81-49E9-8E91-D91E022A6081}">
-  <dimension ref="B1:E3"/>
-  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="2" max="2" width="4.75" customWidth="1"/>
-    <col min="3" max="5" width="10.75" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:5" ht="17.5" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="2" spans="2:5" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B2" s="25" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="2:5" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B3" s="26"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B2:B3"/>
-  </mergeCells>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>